<commit_message>
Graphics revamp: real pixel-art sprites (LPC), village layout, player fix
Replace hand-drawn shapes/emoji with Liberated Pixel Cup sprites for
grass, player, trees, rocks, dungeon/castle walls & floors, chests,
fence/gates, house entrances, altar, and paths, each with a
hand-drawn-fallback if the sprite fails to load.

Player starts in a humble look (blonde hair, simple shirt/pants, no
armor) with soldier+helmet assets kept unused for a future
found-armor mechanic. Fixes a bug where the first composited player
sprite was missing its head/face — the LPC generator's body layer is
headless by design, so the head is now composited in as its own layer.

Also moves the village houses to the four corners with the altar and
a cross of paths at the center, and narrows dungeon/castle walls to
brick only where adjacent to floor (deep rock beyond reads as flat grey).
</commit_message>
<xml_diff>
--- a/valley game design.xlsx
+++ b/valley game design.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tobia\Valley Game\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EBDA6AC7-A7E6-4578-BB73-BA9530382AD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D929F89-420C-4EBC-9E20-46AEA19C1722}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{D62C19FB-41D5-4328-8656-7E243B9A768C}"/>
   </bookViews>
@@ -25,19 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="162">
-  <si>
-    <t>Inventory system</t>
-  </si>
-  <si>
-    <t>storage system</t>
-  </si>
-  <si>
-    <t>crafting system</t>
-  </si>
-  <si>
-    <t>encounter</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="187">
   <si>
     <t>Stats (HP, MP, Strength, Agility, etc.)</t>
   </si>
@@ -144,9 +132,6 @@
     <t>Day/night cycle (optional)</t>
   </si>
   <si>
-    <t>8. NPC &amp; Dialogue System</t>
-  </si>
-  <si>
     <t>Dialogue choices</t>
   </si>
   <si>
@@ -157,9 +142,6 @@
   </si>
   <si>
     <t>Factions (optional)</t>
-  </si>
-  <si>
-    <t>9. Economy System</t>
   </si>
   <si>
     <t>Currency</t>
@@ -732,12 +714,117 @@
   <si>
     <t>This keeps tension high and makes dungeon navigation feel dangerous.</t>
   </si>
+  <si>
+    <t>Monster Zoo</t>
+  </si>
+  <si>
+    <t>gotta collect them all</t>
+  </si>
+  <si>
+    <t>multiple users</t>
+  </si>
+  <si>
+    <t>leaderboard tracker</t>
+  </si>
+  <si>
+    <t>level 1 gather resources</t>
+  </si>
+  <si>
+    <t>starter zone is safe</t>
+  </si>
+  <si>
+    <t>learn to craft</t>
+  </si>
+  <si>
+    <t>NPC &amp; Dialogue System</t>
+  </si>
+  <si>
+    <t>Economy System</t>
+  </si>
+  <si>
+    <t>Dungeons</t>
+  </si>
+  <si>
+    <t>Multi room</t>
+  </si>
+  <si>
+    <t>Place rooms randomly on a grid.</t>
+  </si>
+  <si>
+    <t>Reject overlapping rooms.</t>
+  </si>
+  <si>
+    <t>Connect rooms with corridors.</t>
+  </si>
+  <si>
+    <t>Fill remaining space with walls.</t>
+  </si>
+  <si>
+    <r>
+      <t>Result:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Classic roguelike layout (Binding of Isaac, Shining in the Darkness).</t>
+    </r>
+  </si>
+  <si>
+    <t>Kill mini boss</t>
+  </si>
+  <si>
+    <t>to get key for final room</t>
+  </si>
+  <si>
+    <t>Drop items</t>
+  </si>
+  <si>
+    <t>Show stats allways on screen - hud</t>
+  </si>
+  <si>
+    <t>Death - message</t>
+  </si>
+  <si>
+    <t>reorganise monsters and biomes</t>
+  </si>
+  <si>
+    <t>add NPCs</t>
+  </si>
+  <si>
+    <t>Luigi</t>
+  </si>
+  <si>
+    <t>Eden</t>
+  </si>
+  <si>
+    <t>skill levels</t>
+  </si>
+  <si>
+    <t>Dexterity: Aim, Agility, Construction, Sleight of Hand, Stealth</t>
+  </si>
+  <si>
+    <t>Instinct: Insight, Nature, Perception, Reflex, Will</t>
+  </si>
+  <si>
+    <t>Charisma: Deception, Intimidation, Performance, Persuasion, Seduction</t>
+  </si>
+  <si>
+    <t>Knowledge: Analysis, Lore, Medicine, Science, Technology</t>
+  </si>
+  <si>
+    <t>Strength: Brawling, Fortitude, Power, Stamina, Weaponry</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -769,6 +856,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="7"/>
+      <color rgb="FF333D42"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -796,7 +889,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -815,6 +908,10 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1130,707 +1227,777 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB96D73C-52FA-4CD7-B1C1-EACB155B21E0}">
-  <dimension ref="B3:N137"/>
+  <dimension ref="C6:N137"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="6" max="6" width="41" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="89.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="89.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B3" t="s">
+    <row r="6" spans="3:14" ht="23.5" x14ac:dyDescent="0.35">
+      <c r="C6" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="M6" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="7" spans="3:14" x14ac:dyDescent="0.35">
+      <c r="C7" s="4" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B4" t="s">
+      <c r="F7" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="8" spans="3:14" ht="17.5" x14ac:dyDescent="0.35">
+      <c r="C8" s="2" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B5" t="s">
+      <c r="F8" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="M8" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="9" spans="3:14" x14ac:dyDescent="0.35">
+      <c r="C9" s="2" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="6" spans="2:14" ht="23.5" x14ac:dyDescent="0.35">
-      <c r="B6" t="s">
+      <c r="F9" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="K9" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="10" spans="3:14" x14ac:dyDescent="0.35">
+      <c r="C10" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="K10" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="M10" s="2" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="11" spans="3:14" ht="17.5" x14ac:dyDescent="0.35">
+      <c r="C11" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="K11" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="M11" s="2" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="12" spans="3:14" x14ac:dyDescent="0.35">
+      <c r="C12" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="K12" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="M12" s="2" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="13" spans="3:14" x14ac:dyDescent="0.35">
+      <c r="C13" s="2"/>
+      <c r="F13" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="K13" t="s">
+        <v>88</v>
+      </c>
+      <c r="M13" s="2" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="14" spans="3:14" ht="17.5" x14ac:dyDescent="0.35">
+      <c r="C14" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="M14" s="7" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="15" spans="3:14" ht="23.5" x14ac:dyDescent="0.35">
+      <c r="C15" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="K15" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="M15" s="2"/>
+    </row>
+    <row r="16" spans="3:14" ht="17.5" x14ac:dyDescent="0.35">
+      <c r="C16" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="K16" t="s">
+        <v>90</v>
+      </c>
+      <c r="N16" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="17" spans="3:14" x14ac:dyDescent="0.35">
+      <c r="C17" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="K17" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="N17" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="18" spans="3:14" x14ac:dyDescent="0.35">
+      <c r="C18" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="K18" s="6" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="19" spans="3:14" x14ac:dyDescent="0.35">
+      <c r="C19" s="2"/>
+      <c r="F19" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="K19" s="6" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="20" spans="3:14" ht="17.5" x14ac:dyDescent="0.35">
+      <c r="C20" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="K20" s="6" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="21" spans="3:14" ht="17.5" x14ac:dyDescent="0.35">
+      <c r="C21" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="K21" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="M21" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="22" spans="3:14" x14ac:dyDescent="0.35">
+      <c r="C22" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="K22" t="s">
+        <v>96</v>
+      </c>
+      <c r="M22" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="23" spans="3:14" x14ac:dyDescent="0.35">
+      <c r="C23" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="K23" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="24" spans="3:14" x14ac:dyDescent="0.35">
+      <c r="C24" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="25" spans="3:14" ht="23.5" x14ac:dyDescent="0.35">
+      <c r="C25" s="2"/>
+      <c r="F25" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="K25" s="5" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="26" spans="3:14" ht="17.5" x14ac:dyDescent="0.35">
+      <c r="C26" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F26" s="2"/>
+      <c r="K26" t="s">
+        <v>99</v>
+      </c>
+      <c r="M26" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="27" spans="3:14" ht="17.5" x14ac:dyDescent="0.35">
+      <c r="C27" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="K27" s="6" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="28" spans="3:14" x14ac:dyDescent="0.35">
+      <c r="C28" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="K28" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="M28" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="29" spans="3:14" x14ac:dyDescent="0.35">
+      <c r="C29" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="K29" s="6" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="30" spans="3:14" x14ac:dyDescent="0.35">
+      <c r="C30" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="K30" t="s">
+        <v>103</v>
+      </c>
+      <c r="M30" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="31" spans="3:14" x14ac:dyDescent="0.35">
+      <c r="C31" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="K31" s="2"/>
+      <c r="M31" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="32" spans="3:14" ht="23.5" x14ac:dyDescent="0.35">
+      <c r="K32" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="M32" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="33" spans="3:13" ht="17.5" x14ac:dyDescent="0.35">
+      <c r="C33" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="K33" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="34" spans="3:13" ht="17.5" x14ac:dyDescent="0.35">
+      <c r="C34" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="I6" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="N6" s="5" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="7" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="F7" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="I7" s="2" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="8" spans="2:14" ht="17.5" x14ac:dyDescent="0.35">
-      <c r="F8" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="I8" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="N8" s="1" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="9" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="F9" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="I9" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="N9" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="10" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="F10" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="N10" s="2" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="11" spans="2:14" ht="17.5" x14ac:dyDescent="0.35">
-      <c r="F11" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="I11" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="N11" s="2" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="12" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="F12" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="I12" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="N12" s="2" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="13" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="F13" s="2"/>
-      <c r="I13" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="N13" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="14" spans="2:14" ht="17.5" x14ac:dyDescent="0.35">
-      <c r="F14" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="I14" s="2" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="15" spans="2:14" ht="23.5" x14ac:dyDescent="0.35">
-      <c r="F15" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="N15" s="5" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="16" spans="2:14" ht="17.5" x14ac:dyDescent="0.35">
-      <c r="F16" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="I16" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="N16" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="17" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="F17" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I17" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="N17" s="6" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="18" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="F18" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="I18" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="N18" s="6" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="19" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="F19" s="2"/>
-      <c r="I19" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="N19" s="6" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="20" spans="6:14" ht="17.5" x14ac:dyDescent="0.35">
-      <c r="F20" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="N20" s="6" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="21" spans="6:14" ht="17.5" x14ac:dyDescent="0.35">
-      <c r="F21" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="I21" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="N21" s="6" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="22" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="F22" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I22" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="N22" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="23" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="F23" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="I23" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="N23" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="24" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="F24" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="I24" s="2" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="25" spans="6:14" ht="23.5" x14ac:dyDescent="0.35">
-      <c r="F25" s="2"/>
-      <c r="I25" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="N25" s="5" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="26" spans="6:14" ht="17.5" x14ac:dyDescent="0.35">
-      <c r="F26" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="I26" s="2"/>
-      <c r="N26" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="27" spans="6:14" ht="17.5" x14ac:dyDescent="0.35">
-      <c r="F27" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="I27" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="N27" s="6" t="s">
+      <c r="F34" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="K34" s="2" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="28" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="F28" s="4" t="s">
+    <row r="35" spans="3:13" x14ac:dyDescent="0.35">
+      <c r="C35" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I28" s="2" t="s">
+      <c r="F35" t="s">
+        <v>157</v>
+      </c>
+      <c r="K35" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="M35" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="36" spans="3:13" x14ac:dyDescent="0.35">
+      <c r="C36" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="K36" s="2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="37" spans="3:13" x14ac:dyDescent="0.35">
+      <c r="C37" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="K37" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="38" spans="3:13" ht="52.5" x14ac:dyDescent="0.35">
+      <c r="C38" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="K38" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="M38" s="8" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="39" spans="3:13" ht="52.5" x14ac:dyDescent="0.35">
+      <c r="C39" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K39" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="M39" s="8" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="40" spans="3:13" ht="63" x14ac:dyDescent="0.35">
+      <c r="C40" s="2"/>
+      <c r="K40" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="M40" s="8" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="41" spans="3:13" ht="52.5" x14ac:dyDescent="0.35">
+      <c r="C41" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="K41" t="s">
+        <v>113</v>
+      </c>
+      <c r="M41" s="8" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="42" spans="3:13" ht="63" x14ac:dyDescent="0.35">
+      <c r="C42" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F42" s="2"/>
+      <c r="M42" s="8" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="43" spans="3:13" ht="23.5" x14ac:dyDescent="0.35">
+      <c r="C43" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="K43" s="5" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="44" spans="3:13" x14ac:dyDescent="0.35">
+      <c r="C44" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="F44" s="2"/>
+      <c r="K44" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="45" spans="3:13" x14ac:dyDescent="0.35">
+      <c r="C45" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="F45" t="s">
+        <v>160</v>
+      </c>
+      <c r="K45" s="6" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="46" spans="3:13" x14ac:dyDescent="0.35">
+      <c r="C46" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="F46" t="s">
+        <v>161</v>
+      </c>
+      <c r="K46" s="6" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="47" spans="3:13" x14ac:dyDescent="0.35">
+      <c r="F47" t="s">
+        <v>162</v>
+      </c>
+      <c r="K47" s="6" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="48" spans="3:13" ht="17.5" x14ac:dyDescent="0.35">
+      <c r="C48" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="K48" s="6" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="49" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C49" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="K49" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="50" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C50" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="K50" s="2" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="51" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C51" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="N28" s="6" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="29" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="F29" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="I29" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="N29" s="6" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="30" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="F30" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="I30" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="N30" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="31" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="F31" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="I31" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="N31" s="2"/>
-    </row>
-    <row r="32" spans="6:14" ht="23.5" x14ac:dyDescent="0.35">
-      <c r="N32" s="5" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="33" spans="6:14" ht="17.5" x14ac:dyDescent="0.35">
-      <c r="F33" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="N33" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="34" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="F34" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="N34" s="2" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="35" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="F35" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="N35" s="2" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="36" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="F36" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="N36" s="2" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="37" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="F37" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="N37" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="38" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="F38" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="N38" s="2" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="39" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="F39" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="N39" s="2" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="40" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="F40" s="2"/>
-      <c r="N40" s="2" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="41" spans="6:14" ht="17.5" x14ac:dyDescent="0.35">
-      <c r="F41" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="N41" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="42" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="F42" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="I42" s="2"/>
-    </row>
-    <row r="43" spans="6:14" ht="23.5" x14ac:dyDescent="0.35">
-      <c r="F43" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="N43" s="5" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="44" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="F44" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="I44" s="2"/>
-      <c r="N44" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="45" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="F45" s="2" t="s">
+      <c r="K51" s="2" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="52" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C52" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="N45" s="6" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="46" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="F46" s="2" t="s">
+      <c r="K52" s="2" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="53" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C53" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="N46" s="6" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="47" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="N47" s="6" t="s">
+      <c r="K53" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="48" spans="6:14" ht="17.5" x14ac:dyDescent="0.35">
-      <c r="F48" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="N48" s="6" t="s">
+    <row r="55" spans="3:11" ht="23.5" x14ac:dyDescent="0.35">
+      <c r="C55" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="K55" s="5" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="49" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="F49" s="4" t="s">
+    <row r="56" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C56" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="N49" t="s">
+      <c r="K56" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="50" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="F50" s="4" t="s">
+    <row r="57" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C57" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="N50" s="2" t="s">
+      <c r="K57" s="2" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="51" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="F51" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="N51" s="2" t="s">
+    <row r="58" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C58" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="K58" s="2" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="52" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="F52" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="N52" s="2" t="s">
+    <row r="59" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C59" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="K59" s="2" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="53" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="F53" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="N53" t="s">
+    <row r="60" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="K60" s="2" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="55" spans="6:14" ht="23.5" x14ac:dyDescent="0.35">
-      <c r="F55" s="1" t="s">
+    <row r="61" spans="3:11" ht="17.5" x14ac:dyDescent="0.35">
+      <c r="C61" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="K61" s="2" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="62" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C62" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="N55" s="5" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="56" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="F56" s="2" t="s">
+      <c r="K62" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="63" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C63" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="N56" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="57" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="F57" s="2" t="s">
+      <c r="K63" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="64" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C64" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="N57" s="2" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="58" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="F58" s="2" t="s">
+      <c r="K64" s="2" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="65" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C65" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="N58" s="2" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="59" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="F59" s="2" t="s">
+      <c r="K65" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="66" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C66" s="2"/>
+      <c r="K66" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="67" spans="3:11" ht="17.5" x14ac:dyDescent="0.35">
+      <c r="C67" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="N59" s="2" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="60" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="N60" s="2" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="61" spans="6:14" ht="17.5" x14ac:dyDescent="0.35">
-      <c r="F61" s="1" t="s">
+    </row>
+    <row r="68" spans="3:11" ht="23.5" x14ac:dyDescent="0.35">
+      <c r="C68" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="N61" s="2" t="s">
+      <c r="K68" s="5" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="62" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="F62" s="2" t="s">
+    <row r="69" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C69" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="N62" t="s">
+      <c r="K69" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="63" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="F63" s="2" t="s">
+    <row r="70" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C70" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="N63" s="2" t="s">
+      <c r="K70" s="2" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="64" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="F64" s="2" t="s">
+    <row r="71" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C71" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="N64" s="2" t="s">
+      <c r="K71" s="2" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="65" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="F65" s="2" t="s">
+    <row r="72" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="K72" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="73" spans="3:11" ht="17.5" x14ac:dyDescent="0.35">
+      <c r="C73" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="N65" s="2" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="66" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="F66" s="2"/>
-      <c r="N66" t="s">
+      <c r="K73" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="67" spans="6:14" ht="17.5" x14ac:dyDescent="0.35">
-      <c r="F67" s="1" t="s">
+    <row r="74" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C74" s="2" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="68" spans="6:14" ht="23.5" x14ac:dyDescent="0.35">
-      <c r="F68" s="2" t="s">
+    <row r="75" spans="3:11" ht="23.5" x14ac:dyDescent="0.35">
+      <c r="C75" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="N68" s="5" t="s">
+      <c r="K75" s="5" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="69" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="F69" s="2" t="s">
+    <row r="76" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C76" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="N69" t="s">
+      <c r="K76" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="70" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="F70" s="2" t="s">
+    <row r="77" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C77" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="N70" s="2" t="s">
+      <c r="K77" s="2" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="71" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="F71" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="N71" s="2" t="s">
+    <row r="78" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C78" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="K78" s="2" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="72" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="N72" s="2" t="s">
+    <row r="79" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C79" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="K79" s="2" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="73" spans="6:14" ht="17.5" x14ac:dyDescent="0.35">
-      <c r="F73" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="N73" t="s">
+    <row r="80" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C80" s="2"/>
+      <c r="K80" s="2" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="74" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="F74" s="2" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="75" spans="6:14" ht="23.5" x14ac:dyDescent="0.35">
-      <c r="F75" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="N75" s="5" t="s">
+    <row r="81" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="K81" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="76" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="F76" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="N76" t="s">
+    <row r="82" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C82" s="2"/>
+      <c r="K82" s="2"/>
+    </row>
+    <row r="83" spans="3:11" ht="23.5" x14ac:dyDescent="0.35">
+      <c r="K83" s="5" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="77" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="F77" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="N77" s="2" t="s">
+    <row r="84" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="K84" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="78" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="N78" s="2" t="s">
+    <row r="85" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="K85" s="2" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="79" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="N79" s="2" t="s">
+    <row r="86" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="K86" s="2" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="80" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="F80" s="2"/>
-      <c r="N80" s="2" t="s">
+    <row r="87" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="K87" s="2" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="81" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="N81" t="s">
+    <row r="88" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="K88" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="82" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="F82" s="2"/>
-      <c r="N82" s="2"/>
-    </row>
-    <row r="83" spans="6:14" ht="23.5" x14ac:dyDescent="0.35">
-      <c r="N83" s="5" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="84" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="N84" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="85" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="N85" s="2" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="86" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="N86" s="2" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="87" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="N87" s="2" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="88" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="N88" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="90" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="F90" s="2"/>
-    </row>
-    <row r="91" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="N91" s="2"/>
-    </row>
-    <row r="92" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="F92" s="2"/>
-    </row>
-    <row r="107" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N107" s="2"/>
-    </row>
-    <row r="109" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N109" s="2"/>
-    </row>
-    <row r="111" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N111" s="2"/>
-    </row>
-    <row r="123" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N123" s="2"/>
-    </row>
-    <row r="135" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N135" s="2"/>
-    </row>
-    <row r="137" spans="14:14" x14ac:dyDescent="0.35">
-      <c r="N137" s="2"/>
+    <row r="90" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C90" s="2"/>
+    </row>
+    <row r="91" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="K91" s="2"/>
+    </row>
+    <row r="92" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C92" s="2"/>
+    </row>
+    <row r="107" spans="11:11" x14ac:dyDescent="0.35">
+      <c r="K107" s="2"/>
+    </row>
+    <row r="109" spans="11:11" x14ac:dyDescent="0.35">
+      <c r="K109" s="2"/>
+    </row>
+    <row r="111" spans="11:11" x14ac:dyDescent="0.35">
+      <c r="K111" s="2"/>
+    </row>
+    <row r="123" spans="11:11" x14ac:dyDescent="0.35">
+      <c r="K123" s="2"/>
+    </row>
+    <row r="135" spans="11:11" x14ac:dyDescent="0.35">
+      <c r="K135" s="2"/>
+    </row>
+    <row r="137" spans="11:11" x14ac:dyDescent="0.35">
+      <c r="K137" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>